<commit_message>
Excel Kliniği ücretsiz dosyalar: denetim düzeltmeleri (1. tur)
- DOZ: Özet'in kategori tablosu 12 satır; Kategoriler sayfası, açılır liste ve Başla kapasitesi de 12
  (önceki "20 kategori" iddiası 13.–20. kategoriyi tabloda göstermiyordu); ürün metni "12 kategoriye"
- RİTİM: bugünün satırına çerçeve değil yeşil dolgu ve yazı geliyor; Takip alt başlığı ve ürün metni buna göre

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FcJ9eYFL81XLJVo3qWny3N
</commit_message>
<xml_diff>
--- a/dosyalar/excel-klinigi/ExcelKlinigi_DOZ_Duzenli_Odeme_Takibi.xlsx
+++ b/dosyalar/excel-klinigi/ExcelKlinigi_DOZ_Duzenli_Odeme_Takibi.xlsx
@@ -81,7 +81,7 @@
     <t xml:space="preserve">Kapasite</t>
   </si>
   <si>
-    <t xml:space="preserve">100 ödeme, 20 kategori.</t>
+    <t xml:space="preserve">100 ödeme, 12 kategori.</t>
   </si>
   <si>
     <t xml:space="preserve">RENKLER</t>
@@ -1048,11 +1048,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="18582986"/>
-        <c:axId val="32619560"/>
+        <c:axId val="73785443"/>
+        <c:axId val="44745357"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="18582986"/>
+        <c:axId val="73785443"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1084,7 +1084,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="32619560"/>
+        <c:crossAx val="44745357"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1092,7 +1092,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="32619560"/>
+        <c:axId val="44745357"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1124,7 +1124,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="18582986"/>
+        <c:crossAx val="73785443"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -6101,7 +6101,7 @@
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" error="Listeden seç." errorStyle="stop" errorTitle="Kontrol" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B5:B104" type="list">
-      <formula1>Kategoriler!$A$5:$A$24</formula1>
+      <formula1>Kategoriler!$A$5:$A$16</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -12467,7 +12467,7 @@
     <tabColor rgb="FF1F6F43"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:A24"/>
+  <dimension ref="A1:A16"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
@@ -12539,30 +12539,6 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="12"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="12"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="12"/>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="12"/>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="12"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="12"/>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="12"/>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="12"/>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="12"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>